<commit_message>
Temperature correction to 25degC
</commit_message>
<xml_diff>
--- a/src/hydrofia/hydrofia_ph_template.xlsx
+++ b/src/hydrofia/hydrofia_ph_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20410"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20416"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\mw\git\hydrofia\hydrofia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hydrofia\src\hydrofia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F64928EC-0AC6-4826-A919-F5951EDA7A91}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4CDFA7-4295-4239-8A7F-A40C9380475E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="165" windowWidth="15600" windowHeight="11610" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="170" windowWidth="15600" windowHeight="11610" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rådata" sheetId="4" r:id="rId1"/>
@@ -46,7 +46,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H10" authorId="1" shapeId="0" xr:uid="{21853188-1459-4735-90C6-F9F3174E1258}">
+    <comment ref="J10" authorId="1" shapeId="0" xr:uid="{21853188-1459-4735-90C6-F9F3174E1258}">
       <text>
         <r>
           <rPr>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t>Djup</t>
   </si>
@@ -125,10 +125,16 @@
     <t>C</t>
   </si>
   <si>
-    <t>insitu</t>
+    <t>pH-TOT</t>
   </si>
   <si>
-    <t>pH-TOT</t>
+    <t>labT</t>
+  </si>
+  <si>
+    <t>25degC</t>
+  </si>
+  <si>
+    <t>Lab. Temp</t>
   </si>
 </sst>
 </file>
@@ -394,7 +400,7 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -507,6 +513,16 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -559,9 +575,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>908574</xdr:colOff>
+      <xdr:colOff>905399</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>121875</xdr:rowOff>
+      <xdr:rowOff>125050</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -936,7 +952,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8B184CC-18AA-4DD3-91F3-47A3A5EC6B5D}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -947,32 +963,33 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A1:EF110"/>
-  <sheetFormatPr defaultColWidth="28.7109375" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:EH110"/>
+  <sheetFormatPr defaultColWidth="28.7265625" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="23.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="6.5703125" style="3" customWidth="1"/>
-    <col min="4" max="7" width="7.85546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" style="3" customWidth="1"/>
-    <col min="9" max="17" width="10.7109375" style="3" customWidth="1"/>
-    <col min="18" max="16384" width="28.7109375" style="3"/>
+    <col min="1" max="1" width="15.7265625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="6.54296875" style="3" customWidth="1"/>
+    <col min="4" max="6" width="7.81640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.81640625" style="3" customWidth="1"/>
+    <col min="8" max="9" width="7.81640625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="12.453125" style="3" customWidth="1"/>
+    <col min="11" max="19" width="10.7265625" style="3" customWidth="1"/>
+    <col min="20" max="16384" width="28.7265625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:136" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:138" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2"/>
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="G1" s="32" t="s">
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="H1" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="33"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="33"/>
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
       <c r="R1" s="4"/>
@@ -1094,19 +1111,20 @@
       <c r="ED1" s="4"/>
       <c r="EE1" s="4"/>
       <c r="EF1" s="4"/>
-    </row>
-    <row r="2" spans="1:136" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="G2" s="32" t="s">
+      <c r="EG1" s="4"/>
+      <c r="EH1" s="4"/>
+    </row>
+    <row r="2" spans="1:138" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="H2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="36"/>
-      <c r="I2" s="34"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="34"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
@@ -1228,16 +1246,17 @@
       <c r="ED2" s="4"/>
       <c r="EE2" s="4"/>
       <c r="EF2" s="4"/>
-    </row>
-    <row r="3" spans="1:136" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="35"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
+      <c r="EG2" s="4"/>
+      <c r="EH2" s="4"/>
+    </row>
+    <row r="3" spans="1:138" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="35"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
       <c r="R3" s="4"/>
@@ -1359,8 +1378,10 @@
       <c r="ED3" s="4"/>
       <c r="EE3" s="4"/>
       <c r="EF3" s="4"/>
-    </row>
-    <row r="4" spans="1:136" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="EG3" s="4"/>
+      <c r="EH3" s="4"/>
+    </row>
+    <row r="4" spans="1:138" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>1</v>
       </c>
@@ -1368,10 +1389,9 @@
       <c r="C4" s="25"/>
       <c r="D4" s="25"/>
       <c r="E4" s="25"/>
-      <c r="G4" s="23"/>
       <c r="H4" s="23"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
@@ -1493,27 +1513,29 @@
       <c r="ED4" s="4"/>
       <c r="EE4" s="4"/>
       <c r="EF4" s="4"/>
-    </row>
-    <row r="5" spans="1:136" s="1" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="EG4" s="4"/>
+      <c r="EH4" s="4"/>
+    </row>
+    <row r="5" spans="1:138" s="1" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="29" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="26"/>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="43"/>
-      <c r="E5" s="42" t="s">
+      <c r="D5" s="46"/>
+      <c r="E5" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="43"/>
-      <c r="G5" s="41" t="s">
+      <c r="F5" s="46"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="41"/>
-      <c r="I5" s="6"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="6"/>
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
@@ -1635,19 +1657,21 @@
       <c r="ED5" s="7"/>
       <c r="EE5" s="7"/>
       <c r="EF5" s="7"/>
-    </row>
-    <row r="6" spans="1:136" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="EG5" s="7"/>
+      <c r="EH5" s="7"/>
+    </row>
+    <row r="6" spans="1:138" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="28"/>
       <c r="B6" s="20"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="8"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="43"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="8"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="4"/>
@@ -1769,42 +1793,50 @@
       <c r="ED6" s="4"/>
       <c r="EE6" s="4"/>
       <c r="EF6" s="4"/>
-    </row>
-    <row r="7" spans="1:136" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="EG6" s="4"/>
+      <c r="EH6" s="4"/>
+    </row>
+    <row r="7" spans="1:138" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="28"/>
       <c r="B7" s="20"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="40"/>
-    </row>
-    <row r="8" spans="1:136" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+    </row>
+    <row r="8" spans="1:138" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="28"/>
       <c r="B8" s="20"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-    </row>
-    <row r="9" spans="1:136" s="4" customFormat="1" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+    </row>
+    <row r="9" spans="1:138" s="4" customFormat="1" ht="5.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="10"/>
-      <c r="G9" s="11"/>
+      <c r="G9" s="10"/>
       <c r="H9" s="11"/>
-    </row>
-    <row r="10" spans="1:136" s="4" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A10" s="38" t="s">
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+    </row>
+    <row r="10" spans="1:138" s="4" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="41" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="19" t="s">
@@ -1820,15 +1852,21 @@
         <v>12</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
-      <c r="H10" s="38" t="s">
+      <c r="H10" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" s="41" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:136" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="39"/>
-      <c r="B11" s="39"/>
+    <row r="11" spans="1:138" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="42"/>
+      <c r="B11" s="42"/>
       <c r="C11" s="14" t="s">
         <v>5</v>
       </c>
@@ -1839,1010 +1877,1214 @@
       <c r="F11" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="15" t="s">
-        <v>16</v>
+      <c r="G11" s="27" t="s">
+        <v>15</v>
       </c>
-      <c r="H11" s="39"/>
-    </row>
-    <row r="12" spans="1:136" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H11" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="42"/>
+    </row>
+    <row r="12" spans="1:138" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="21"/>
       <c r="B12" s="30"/>
       <c r="C12" s="21"/>
       <c r="D12" s="21"/>
       <c r="E12" s="21"/>
       <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
+      <c r="G12" s="30"/>
       <c r="H12" s="21"/>
-    </row>
-    <row r="13" spans="1:136" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I12" s="30"/>
+      <c r="J12" s="21"/>
+    </row>
+    <row r="13" spans="1:138" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="21"/>
       <c r="B13" s="30"/>
       <c r="C13" s="21"/>
       <c r="D13" s="21"/>
       <c r="E13" s="21"/>
       <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
+      <c r="G13" s="30"/>
       <c r="H13" s="21"/>
-    </row>
-    <row r="14" spans="1:136" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I13" s="30"/>
+      <c r="J13" s="21"/>
+    </row>
+    <row r="14" spans="1:138" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="21"/>
       <c r="B14" s="30"/>
       <c r="C14" s="21"/>
       <c r="D14" s="21"/>
       <c r="E14" s="21"/>
       <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
+      <c r="G14" s="30"/>
       <c r="H14" s="21"/>
-    </row>
-    <row r="15" spans="1:136" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I14" s="30"/>
+      <c r="J14" s="21"/>
+    </row>
+    <row r="15" spans="1:138" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="21"/>
       <c r="B15" s="30"/>
       <c r="C15" s="21"/>
       <c r="D15" s="21"/>
       <c r="E15" s="21"/>
       <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
+      <c r="G15" s="30"/>
       <c r="H15" s="21"/>
-    </row>
-    <row r="16" spans="1:136" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I15" s="30"/>
+      <c r="J15" s="21"/>
+    </row>
+    <row r="16" spans="1:138" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="21"/>
       <c r="B16" s="30"/>
       <c r="C16" s="21"/>
       <c r="D16" s="21"/>
       <c r="E16" s="21"/>
       <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
+      <c r="G16" s="30"/>
       <c r="H16" s="21"/>
-    </row>
-    <row r="17" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I16" s="30"/>
+      <c r="J16" s="21"/>
+    </row>
+    <row r="17" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="21"/>
       <c r="B17" s="30"/>
       <c r="C17" s="21"/>
       <c r="D17" s="21"/>
       <c r="E17" s="21"/>
       <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
+      <c r="G17" s="30"/>
       <c r="H17" s="21"/>
-    </row>
-    <row r="18" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I17" s="30"/>
+      <c r="J17" s="21"/>
+    </row>
+    <row r="18" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="21"/>
       <c r="B18" s="30"/>
       <c r="C18" s="21"/>
       <c r="D18" s="21"/>
       <c r="E18" s="21"/>
       <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
+      <c r="G18" s="30"/>
       <c r="H18" s="21"/>
-    </row>
-    <row r="19" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I18" s="30"/>
+      <c r="J18" s="21"/>
+    </row>
+    <row r="19" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="21"/>
       <c r="B19" s="30"/>
       <c r="C19" s="21"/>
       <c r="D19" s="21"/>
       <c r="E19" s="21"/>
       <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
+      <c r="G19" s="30"/>
       <c r="H19" s="21"/>
-    </row>
-    <row r="20" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I19" s="30"/>
+      <c r="J19" s="21"/>
+    </row>
+    <row r="20" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="21"/>
       <c r="B20" s="30"/>
       <c r="C20" s="21"/>
       <c r="D20" s="21"/>
       <c r="E20" s="21"/>
       <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
+      <c r="G20" s="30"/>
       <c r="H20" s="21"/>
-    </row>
-    <row r="21" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I20" s="30"/>
+      <c r="J20" s="21"/>
+    </row>
+    <row r="21" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="21"/>
       <c r="B21" s="30"/>
       <c r="C21" s="21"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
       <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
+      <c r="G21" s="30"/>
       <c r="H21" s="21"/>
-    </row>
-    <row r="22" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I21" s="30"/>
+      <c r="J21" s="21"/>
+    </row>
+    <row r="22" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="21"/>
       <c r="B22" s="30"/>
       <c r="C22" s="21"/>
       <c r="D22" s="21"/>
       <c r="E22" s="21"/>
       <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
+      <c r="G22" s="30"/>
       <c r="H22" s="21"/>
-    </row>
-    <row r="23" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I22" s="30"/>
+      <c r="J22" s="21"/>
+    </row>
+    <row r="23" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="21"/>
       <c r="B23" s="30"/>
       <c r="C23" s="21"/>
       <c r="D23" s="21"/>
       <c r="E23" s="21"/>
       <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
+      <c r="G23" s="30"/>
       <c r="H23" s="21"/>
-    </row>
-    <row r="24" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I23" s="30"/>
+      <c r="J23" s="21"/>
+    </row>
+    <row r="24" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="21"/>
       <c r="B24" s="30"/>
       <c r="C24" s="21"/>
       <c r="D24" s="21"/>
       <c r="E24" s="21"/>
       <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
+      <c r="G24" s="30"/>
       <c r="H24" s="21"/>
-    </row>
-    <row r="25" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I24" s="30"/>
+      <c r="J24" s="21"/>
+    </row>
+    <row r="25" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="21"/>
       <c r="B25" s="30"/>
       <c r="C25" s="21"/>
       <c r="D25" s="21"/>
       <c r="E25" s="21"/>
       <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
+      <c r="G25" s="30"/>
       <c r="H25" s="21"/>
-    </row>
-    <row r="26" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I25" s="30"/>
+      <c r="J25" s="21"/>
+    </row>
+    <row r="26" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="21"/>
       <c r="B26" s="30"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
       <c r="E26" s="21"/>
       <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
+      <c r="G26" s="30"/>
       <c r="H26" s="21"/>
-    </row>
-    <row r="27" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I26" s="30"/>
+      <c r="J26" s="21"/>
+    </row>
+    <row r="27" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="21"/>
       <c r="B27" s="30"/>
       <c r="C27" s="21"/>
       <c r="D27" s="21"/>
       <c r="E27" s="21"/>
       <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
+      <c r="G27" s="30"/>
       <c r="H27" s="21"/>
-    </row>
-    <row r="28" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I27" s="30"/>
+      <c r="J27" s="21"/>
+    </row>
+    <row r="28" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="21"/>
       <c r="B28" s="30"/>
       <c r="C28" s="21"/>
       <c r="D28" s="21"/>
       <c r="E28" s="21"/>
       <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
+      <c r="G28" s="30"/>
       <c r="H28" s="21"/>
-    </row>
-    <row r="29" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I28" s="30"/>
+      <c r="J28" s="21"/>
+    </row>
+    <row r="29" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="21"/>
       <c r="B29" s="30"/>
       <c r="C29" s="21"/>
       <c r="D29" s="21"/>
       <c r="E29" s="21"/>
       <c r="F29" s="21"/>
-      <c r="G29" s="21"/>
+      <c r="G29" s="30"/>
       <c r="H29" s="21"/>
-    </row>
-    <row r="30" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I29" s="30"/>
+      <c r="J29" s="21"/>
+    </row>
+    <row r="30" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="21"/>
       <c r="B30" s="30"/>
       <c r="C30" s="21"/>
       <c r="D30" s="21"/>
       <c r="E30" s="21"/>
       <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
+      <c r="G30" s="30"/>
       <c r="H30" s="21"/>
-    </row>
-    <row r="31" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I30" s="30"/>
+      <c r="J30" s="21"/>
+    </row>
+    <row r="31" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="21"/>
       <c r="B31" s="30"/>
       <c r="C31" s="21"/>
       <c r="D31" s="21"/>
       <c r="E31" s="21"/>
       <c r="F31" s="21"/>
-      <c r="G31" s="21"/>
+      <c r="G31" s="30"/>
       <c r="H31" s="21"/>
-    </row>
-    <row r="32" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I31" s="30"/>
+      <c r="J31" s="21"/>
+    </row>
+    <row r="32" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="21"/>
       <c r="B32" s="30"/>
       <c r="C32" s="21"/>
       <c r="D32" s="21"/>
       <c r="E32" s="21"/>
       <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
+      <c r="G32" s="30"/>
       <c r="H32" s="21"/>
-    </row>
-    <row r="33" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I32" s="30"/>
+      <c r="J32" s="21"/>
+    </row>
+    <row r="33" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="21"/>
       <c r="B33" s="30"/>
       <c r="C33" s="21"/>
       <c r="D33" s="21"/>
       <c r="E33" s="21"/>
       <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
+      <c r="G33" s="30"/>
       <c r="H33" s="21"/>
-    </row>
-    <row r="34" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I33" s="30"/>
+      <c r="J33" s="21"/>
+    </row>
+    <row r="34" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="21"/>
       <c r="B34" s="30"/>
       <c r="C34" s="21"/>
       <c r="D34" s="21"/>
       <c r="E34" s="21"/>
       <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
+      <c r="G34" s="30"/>
       <c r="H34" s="21"/>
-    </row>
-    <row r="35" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I34" s="30"/>
+      <c r="J34" s="21"/>
+    </row>
+    <row r="35" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="21"/>
       <c r="B35" s="30"/>
       <c r="C35" s="21"/>
       <c r="D35" s="21"/>
       <c r="E35" s="21"/>
       <c r="F35" s="21"/>
-      <c r="G35" s="21"/>
+      <c r="G35" s="30"/>
       <c r="H35" s="21"/>
-    </row>
-    <row r="36" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I35" s="30"/>
+      <c r="J35" s="21"/>
+    </row>
+    <row r="36" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="21"/>
       <c r="B36" s="30"/>
       <c r="C36" s="21"/>
       <c r="D36" s="21"/>
       <c r="E36" s="21"/>
       <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
+      <c r="G36" s="30"/>
       <c r="H36" s="21"/>
-    </row>
-    <row r="37" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I36" s="30"/>
+      <c r="J36" s="21"/>
+    </row>
+    <row r="37" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="21"/>
       <c r="B37" s="30"/>
       <c r="C37" s="21"/>
       <c r="D37" s="21"/>
       <c r="E37" s="21"/>
       <c r="F37" s="21"/>
-      <c r="G37" s="21"/>
+      <c r="G37" s="30"/>
       <c r="H37" s="21"/>
-    </row>
-    <row r="38" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I37" s="30"/>
+      <c r="J37" s="21"/>
+    </row>
+    <row r="38" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="21"/>
       <c r="B38" s="30"/>
       <c r="C38" s="21"/>
       <c r="D38" s="21"/>
       <c r="E38" s="21"/>
       <c r="F38" s="21"/>
-      <c r="G38" s="21"/>
+      <c r="G38" s="30"/>
       <c r="H38" s="21"/>
-    </row>
-    <row r="39" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I38" s="30"/>
+      <c r="J38" s="21"/>
+    </row>
+    <row r="39" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="21"/>
       <c r="B39" s="30"/>
       <c r="C39" s="21"/>
       <c r="D39" s="21"/>
       <c r="E39" s="21"/>
       <c r="F39" s="21"/>
-      <c r="G39" s="21"/>
+      <c r="G39" s="30"/>
       <c r="H39" s="21"/>
-    </row>
-    <row r="40" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I39" s="30"/>
+      <c r="J39" s="21"/>
+    </row>
+    <row r="40" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="21"/>
       <c r="B40" s="30"/>
       <c r="C40" s="21"/>
       <c r="D40" s="21"/>
       <c r="E40" s="21"/>
       <c r="F40" s="21"/>
-      <c r="G40" s="21"/>
+      <c r="G40" s="30"/>
       <c r="H40" s="21"/>
-    </row>
-    <row r="41" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I40" s="30"/>
+      <c r="J40" s="21"/>
+    </row>
+    <row r="41" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="21"/>
       <c r="B41" s="30"/>
       <c r="C41" s="21"/>
       <c r="D41" s="21"/>
       <c r="E41" s="21"/>
       <c r="F41" s="21"/>
-      <c r="G41" s="21"/>
+      <c r="G41" s="30"/>
       <c r="H41" s="21"/>
-    </row>
-    <row r="42" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I41" s="30"/>
+      <c r="J41" s="21"/>
+    </row>
+    <row r="42" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="21"/>
       <c r="B42" s="30"/>
       <c r="C42" s="21"/>
       <c r="D42" s="21"/>
       <c r="E42" s="21"/>
       <c r="F42" s="21"/>
-      <c r="G42" s="21"/>
+      <c r="G42" s="30"/>
       <c r="H42" s="21"/>
-    </row>
-    <row r="43" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I42" s="30"/>
+      <c r="J42" s="21"/>
+    </row>
+    <row r="43" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="21"/>
       <c r="B43" s="30"/>
       <c r="C43" s="21"/>
       <c r="D43" s="21"/>
       <c r="E43" s="21"/>
       <c r="F43" s="21"/>
-      <c r="G43" s="21"/>
+      <c r="G43" s="30"/>
       <c r="H43" s="21"/>
-    </row>
-    <row r="44" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I43" s="30"/>
+      <c r="J43" s="21"/>
+    </row>
+    <row r="44" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="21"/>
       <c r="B44" s="30"/>
       <c r="C44" s="21"/>
       <c r="D44" s="21"/>
       <c r="E44" s="21"/>
       <c r="F44" s="21"/>
-      <c r="G44" s="21"/>
+      <c r="G44" s="30"/>
       <c r="H44" s="21"/>
-    </row>
-    <row r="45" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I44" s="30"/>
+      <c r="J44" s="21"/>
+    </row>
+    <row r="45" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="21"/>
       <c r="B45" s="30"/>
       <c r="C45" s="21"/>
       <c r="D45" s="21"/>
       <c r="E45" s="21"/>
       <c r="F45" s="21"/>
-      <c r="G45" s="21"/>
+      <c r="G45" s="30"/>
       <c r="H45" s="21"/>
-    </row>
-    <row r="46" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I45" s="30"/>
+      <c r="J45" s="21"/>
+    </row>
+    <row r="46" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="21"/>
       <c r="B46" s="30"/>
       <c r="C46" s="21"/>
       <c r="D46" s="21"/>
       <c r="E46" s="21"/>
       <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
+      <c r="G46" s="30"/>
       <c r="H46" s="21"/>
-    </row>
-    <row r="47" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I46" s="30"/>
+      <c r="J46" s="21"/>
+    </row>
+    <row r="47" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="21"/>
       <c r="B47" s="30"/>
       <c r="C47" s="21"/>
       <c r="D47" s="21"/>
       <c r="E47" s="21"/>
       <c r="F47" s="21"/>
-      <c r="G47" s="21"/>
+      <c r="G47" s="30"/>
       <c r="H47" s="21"/>
-    </row>
-    <row r="48" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I47" s="30"/>
+      <c r="J47" s="21"/>
+    </row>
+    <row r="48" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="21"/>
       <c r="B48" s="30"/>
       <c r="C48" s="21"/>
       <c r="D48" s="21"/>
       <c r="E48" s="21"/>
       <c r="F48" s="21"/>
-      <c r="G48" s="21"/>
+      <c r="G48" s="30"/>
       <c r="H48" s="21"/>
-    </row>
-    <row r="49" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I48" s="30"/>
+      <c r="J48" s="21"/>
+    </row>
+    <row r="49" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="21"/>
       <c r="B49" s="30"/>
       <c r="C49" s="21"/>
       <c r="D49" s="21"/>
       <c r="E49" s="21"/>
       <c r="F49" s="21"/>
-      <c r="G49" s="21"/>
+      <c r="G49" s="30"/>
       <c r="H49" s="21"/>
-    </row>
-    <row r="50" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I49" s="30"/>
+      <c r="J49" s="21"/>
+    </row>
+    <row r="50" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="21"/>
       <c r="B50" s="30"/>
       <c r="C50" s="21"/>
       <c r="D50" s="21"/>
       <c r="E50" s="21"/>
       <c r="F50" s="21"/>
-      <c r="G50" s="21"/>
+      <c r="G50" s="30"/>
       <c r="H50" s="21"/>
-    </row>
-    <row r="51" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I50" s="30"/>
+      <c r="J50" s="21"/>
+    </row>
+    <row r="51" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="21"/>
       <c r="B51" s="30"/>
       <c r="C51" s="21"/>
       <c r="D51" s="21"/>
       <c r="E51" s="21"/>
       <c r="F51" s="21"/>
-      <c r="G51" s="21"/>
+      <c r="G51" s="30"/>
       <c r="H51" s="21"/>
-    </row>
-    <row r="52" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I51" s="30"/>
+      <c r="J51" s="21"/>
+    </row>
+    <row r="52" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="21"/>
       <c r="B52" s="30"/>
       <c r="C52" s="21"/>
       <c r="D52" s="21"/>
       <c r="E52" s="21"/>
       <c r="F52" s="21"/>
-      <c r="G52" s="21"/>
+      <c r="G52" s="30"/>
       <c r="H52" s="21"/>
-    </row>
-    <row r="53" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I52" s="30"/>
+      <c r="J52" s="21"/>
+    </row>
+    <row r="53" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="21"/>
       <c r="B53" s="30"/>
       <c r="C53" s="21"/>
       <c r="D53" s="21"/>
       <c r="E53" s="21"/>
       <c r="F53" s="21"/>
-      <c r="G53" s="21"/>
+      <c r="G53" s="30"/>
       <c r="H53" s="21"/>
-    </row>
-    <row r="54" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I53" s="30"/>
+      <c r="J53" s="21"/>
+    </row>
+    <row r="54" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="21"/>
       <c r="B54" s="30"/>
       <c r="C54" s="21"/>
       <c r="D54" s="21"/>
       <c r="E54" s="21"/>
       <c r="F54" s="21"/>
-      <c r="G54" s="21"/>
+      <c r="G54" s="30"/>
       <c r="H54" s="21"/>
-    </row>
-    <row r="55" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I54" s="30"/>
+      <c r="J54" s="21"/>
+    </row>
+    <row r="55" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="21"/>
       <c r="B55" s="30"/>
       <c r="C55" s="21"/>
       <c r="D55" s="21"/>
       <c r="E55" s="21"/>
       <c r="F55" s="21"/>
-      <c r="G55" s="21"/>
+      <c r="G55" s="30"/>
       <c r="H55" s="21"/>
-    </row>
-    <row r="56" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I55" s="30"/>
+      <c r="J55" s="21"/>
+    </row>
+    <row r="56" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="21"/>
       <c r="B56" s="30"/>
       <c r="C56" s="21"/>
       <c r="D56" s="21"/>
       <c r="E56" s="21"/>
       <c r="F56" s="21"/>
-      <c r="G56" s="21"/>
+      <c r="G56" s="30"/>
       <c r="H56" s="21"/>
-    </row>
-    <row r="57" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I56" s="30"/>
+      <c r="J56" s="21"/>
+    </row>
+    <row r="57" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="21"/>
       <c r="B57" s="30"/>
       <c r="C57" s="21"/>
       <c r="D57" s="21"/>
       <c r="E57" s="21"/>
       <c r="F57" s="21"/>
-      <c r="G57" s="21"/>
+      <c r="G57" s="30"/>
       <c r="H57" s="21"/>
-    </row>
-    <row r="58" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I57" s="30"/>
+      <c r="J57" s="21"/>
+    </row>
+    <row r="58" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="21"/>
       <c r="B58" s="30"/>
       <c r="C58" s="21"/>
       <c r="D58" s="21"/>
       <c r="E58" s="21"/>
       <c r="F58" s="21"/>
-      <c r="G58" s="21"/>
+      <c r="G58" s="30"/>
       <c r="H58" s="21"/>
-    </row>
-    <row r="59" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I58" s="30"/>
+      <c r="J58" s="21"/>
+    </row>
+    <row r="59" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="21"/>
       <c r="B59" s="30"/>
       <c r="C59" s="21"/>
       <c r="D59" s="21"/>
       <c r="E59" s="21"/>
       <c r="F59" s="21"/>
-      <c r="G59" s="21"/>
+      <c r="G59" s="30"/>
       <c r="H59" s="21"/>
-    </row>
-    <row r="60" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I59" s="30"/>
+      <c r="J59" s="21"/>
+    </row>
+    <row r="60" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="21"/>
       <c r="B60" s="30"/>
       <c r="C60" s="21"/>
       <c r="D60" s="21"/>
       <c r="E60" s="21"/>
       <c r="F60" s="21"/>
-      <c r="G60" s="21"/>
+      <c r="G60" s="30"/>
       <c r="H60" s="21"/>
-    </row>
-    <row r="61" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I60" s="30"/>
+      <c r="J60" s="21"/>
+    </row>
+    <row r="61" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="21"/>
       <c r="B61" s="30"/>
       <c r="C61" s="21"/>
       <c r="D61" s="21"/>
       <c r="E61" s="21"/>
       <c r="F61" s="21"/>
-      <c r="G61" s="21"/>
+      <c r="G61" s="30"/>
       <c r="H61" s="21"/>
-    </row>
-    <row r="62" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I61" s="30"/>
+      <c r="J61" s="21"/>
+    </row>
+    <row r="62" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="21"/>
       <c r="B62" s="30"/>
       <c r="C62" s="21"/>
       <c r="D62" s="21"/>
       <c r="E62" s="21"/>
       <c r="F62" s="21"/>
-      <c r="G62" s="21"/>
+      <c r="G62" s="30"/>
       <c r="H62" s="21"/>
-    </row>
-    <row r="63" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I62" s="30"/>
+      <c r="J62" s="21"/>
+    </row>
+    <row r="63" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="21"/>
       <c r="B63" s="30"/>
       <c r="C63" s="21"/>
       <c r="D63" s="21"/>
       <c r="E63" s="21"/>
       <c r="F63" s="21"/>
-      <c r="G63" s="21"/>
+      <c r="G63" s="30"/>
       <c r="H63" s="21"/>
-    </row>
-    <row r="64" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I63" s="30"/>
+      <c r="J63" s="21"/>
+    </row>
+    <row r="64" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="21"/>
       <c r="B64" s="30"/>
       <c r="C64" s="21"/>
       <c r="D64" s="21"/>
       <c r="E64" s="21"/>
       <c r="F64" s="21"/>
-      <c r="G64" s="21"/>
+      <c r="G64" s="30"/>
       <c r="H64" s="21"/>
-    </row>
-    <row r="65" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I64" s="30"/>
+      <c r="J64" s="21"/>
+    </row>
+    <row r="65" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="21"/>
       <c r="B65" s="30"/>
       <c r="C65" s="21"/>
       <c r="D65" s="21"/>
       <c r="E65" s="21"/>
       <c r="F65" s="21"/>
-      <c r="G65" s="21"/>
+      <c r="G65" s="30"/>
       <c r="H65" s="21"/>
-    </row>
-    <row r="66" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I65" s="30"/>
+      <c r="J65" s="21"/>
+    </row>
+    <row r="66" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="21"/>
       <c r="B66" s="30"/>
       <c r="C66" s="21"/>
       <c r="D66" s="21"/>
       <c r="E66" s="21"/>
       <c r="F66" s="21"/>
-      <c r="G66" s="21"/>
+      <c r="G66" s="30"/>
       <c r="H66" s="21"/>
-    </row>
-    <row r="67" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I66" s="30"/>
+      <c r="J66" s="21"/>
+    </row>
+    <row r="67" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="21"/>
       <c r="B67" s="30"/>
       <c r="C67" s="21"/>
       <c r="D67" s="21"/>
       <c r="E67" s="21"/>
       <c r="F67" s="21"/>
-      <c r="G67" s="21"/>
+      <c r="G67" s="30"/>
       <c r="H67" s="21"/>
-    </row>
-    <row r="68" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I67" s="30"/>
+      <c r="J67" s="21"/>
+    </row>
+    <row r="68" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="21"/>
       <c r="B68" s="30"/>
       <c r="C68" s="21"/>
       <c r="D68" s="21"/>
       <c r="E68" s="21"/>
       <c r="F68" s="21"/>
-      <c r="G68" s="21"/>
+      <c r="G68" s="30"/>
       <c r="H68" s="21"/>
-    </row>
-    <row r="69" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I68" s="30"/>
+      <c r="J68" s="21"/>
+    </row>
+    <row r="69" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="21"/>
       <c r="B69" s="30"/>
       <c r="C69" s="21"/>
       <c r="D69" s="21"/>
       <c r="E69" s="21"/>
       <c r="F69" s="21"/>
-      <c r="G69" s="21"/>
+      <c r="G69" s="30"/>
       <c r="H69" s="21"/>
-    </row>
-    <row r="70" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I69" s="30"/>
+      <c r="J69" s="21"/>
+    </row>
+    <row r="70" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="21"/>
       <c r="B70" s="30"/>
       <c r="C70" s="21"/>
       <c r="D70" s="21"/>
       <c r="E70" s="21"/>
       <c r="F70" s="21"/>
-      <c r="G70" s="21"/>
+      <c r="G70" s="30"/>
       <c r="H70" s="21"/>
-    </row>
-    <row r="71" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I70" s="30"/>
+      <c r="J70" s="21"/>
+    </row>
+    <row r="71" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="21"/>
       <c r="B71" s="30"/>
       <c r="C71" s="21"/>
       <c r="D71" s="21"/>
       <c r="E71" s="21"/>
       <c r="F71" s="21"/>
-      <c r="G71" s="21"/>
+      <c r="G71" s="30"/>
       <c r="H71" s="21"/>
-    </row>
-    <row r="72" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I71" s="30"/>
+      <c r="J71" s="21"/>
+    </row>
+    <row r="72" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="21"/>
       <c r="B72" s="30"/>
       <c r="C72" s="21"/>
       <c r="D72" s="21"/>
       <c r="E72" s="21"/>
       <c r="F72" s="21"/>
-      <c r="G72" s="21"/>
+      <c r="G72" s="30"/>
       <c r="H72" s="21"/>
-    </row>
-    <row r="73" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I72" s="30"/>
+      <c r="J72" s="21"/>
+    </row>
+    <row r="73" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="21"/>
       <c r="B73" s="30"/>
       <c r="C73" s="21"/>
       <c r="D73" s="21"/>
       <c r="E73" s="21"/>
       <c r="F73" s="21"/>
-      <c r="G73" s="21"/>
+      <c r="G73" s="30"/>
       <c r="H73" s="21"/>
-    </row>
-    <row r="74" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I73" s="30"/>
+      <c r="J73" s="21"/>
+    </row>
+    <row r="74" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="21"/>
       <c r="B74" s="30"/>
       <c r="C74" s="21"/>
       <c r="D74" s="21"/>
       <c r="E74" s="21"/>
       <c r="F74" s="21"/>
-      <c r="G74" s="21"/>
+      <c r="G74" s="30"/>
       <c r="H74" s="21"/>
-    </row>
-    <row r="75" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I74" s="30"/>
+      <c r="J74" s="21"/>
+    </row>
+    <row r="75" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="21"/>
       <c r="B75" s="30"/>
       <c r="C75" s="21"/>
       <c r="D75" s="21"/>
       <c r="E75" s="21"/>
       <c r="F75" s="21"/>
-      <c r="G75" s="21"/>
+      <c r="G75" s="30"/>
       <c r="H75" s="21"/>
-    </row>
-    <row r="76" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I75" s="30"/>
+      <c r="J75" s="21"/>
+    </row>
+    <row r="76" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="21"/>
       <c r="B76" s="30"/>
       <c r="C76" s="21"/>
       <c r="D76" s="21"/>
       <c r="E76" s="21"/>
       <c r="F76" s="21"/>
-      <c r="G76" s="21"/>
+      <c r="G76" s="30"/>
       <c r="H76" s="21"/>
-    </row>
-    <row r="77" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I76" s="30"/>
+      <c r="J76" s="21"/>
+    </row>
+    <row r="77" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="21"/>
       <c r="B77" s="30"/>
       <c r="C77" s="21"/>
       <c r="D77" s="21"/>
       <c r="E77" s="21"/>
       <c r="F77" s="21"/>
-      <c r="G77" s="21"/>
+      <c r="G77" s="30"/>
       <c r="H77" s="21"/>
-    </row>
-    <row r="78" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I77" s="30"/>
+      <c r="J77" s="21"/>
+    </row>
+    <row r="78" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="21"/>
       <c r="B78" s="30"/>
       <c r="C78" s="21"/>
       <c r="D78" s="21"/>
       <c r="E78" s="21"/>
       <c r="F78" s="21"/>
-      <c r="G78" s="21"/>
+      <c r="G78" s="30"/>
       <c r="H78" s="21"/>
-    </row>
-    <row r="79" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I78" s="30"/>
+      <c r="J78" s="21"/>
+    </row>
+    <row r="79" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="21"/>
       <c r="B79" s="30"/>
       <c r="C79" s="21"/>
       <c r="D79" s="21"/>
       <c r="E79" s="21"/>
       <c r="F79" s="21"/>
-      <c r="G79" s="21"/>
+      <c r="G79" s="30"/>
       <c r="H79" s="21"/>
-    </row>
-    <row r="80" spans="1:8" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I79" s="30"/>
+      <c r="J79" s="21"/>
+    </row>
+    <row r="80" spans="1:10" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="21"/>
       <c r="B80" s="30"/>
       <c r="C80" s="21"/>
       <c r="D80" s="21"/>
       <c r="E80" s="21"/>
       <c r="F80" s="21"/>
-      <c r="G80" s="21"/>
+      <c r="G80" s="30"/>
       <c r="H80" s="21"/>
-    </row>
-    <row r="81" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I80" s="30"/>
+      <c r="J80" s="21"/>
+    </row>
+    <row r="81" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="16"/>
       <c r="B81" s="31"/>
       <c r="C81" s="22"/>
       <c r="D81" s="22"/>
       <c r="E81" s="16"/>
       <c r="F81" s="22"/>
-      <c r="G81" s="22"/>
+      <c r="G81" s="31"/>
       <c r="H81" s="22"/>
-    </row>
-    <row r="82" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I81" s="31"/>
+      <c r="J81" s="22"/>
+    </row>
+    <row r="82" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="16"/>
       <c r="B82" s="31"/>
       <c r="C82" s="22"/>
       <c r="D82" s="22"/>
       <c r="E82" s="16"/>
       <c r="F82" s="22"/>
-      <c r="G82" s="22"/>
+      <c r="G82" s="31"/>
       <c r="H82" s="22"/>
-    </row>
-    <row r="83" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I82" s="31"/>
+      <c r="J82" s="22"/>
+    </row>
+    <row r="83" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="16"/>
       <c r="B83" s="31"/>
       <c r="C83" s="22"/>
       <c r="D83" s="22"/>
       <c r="E83" s="16"/>
       <c r="F83" s="22"/>
-      <c r="G83" s="22"/>
+      <c r="G83" s="31"/>
       <c r="H83" s="22"/>
-    </row>
-    <row r="84" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I83" s="31"/>
+      <c r="J83" s="22"/>
+    </row>
+    <row r="84" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="16"/>
       <c r="B84" s="31"/>
       <c r="C84" s="22"/>
       <c r="D84" s="22"/>
       <c r="E84" s="16"/>
       <c r="F84" s="22"/>
-      <c r="G84" s="22"/>
+      <c r="G84" s="31"/>
       <c r="H84" s="22"/>
-    </row>
-    <row r="85" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I84" s="31"/>
+      <c r="J84" s="22"/>
+    </row>
+    <row r="85" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="16"/>
       <c r="B85" s="31"/>
       <c r="C85" s="22"/>
       <c r="D85" s="22"/>
       <c r="E85" s="16"/>
       <c r="F85" s="22"/>
-      <c r="G85" s="22"/>
+      <c r="G85" s="31"/>
       <c r="H85" s="22"/>
-    </row>
-    <row r="86" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I85" s="31"/>
+      <c r="J85" s="22"/>
+    </row>
+    <row r="86" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="16"/>
       <c r="B86" s="31"/>
       <c r="C86" s="22"/>
       <c r="D86" s="22"/>
       <c r="E86" s="16"/>
       <c r="F86" s="22"/>
-      <c r="G86" s="22"/>
+      <c r="G86" s="31"/>
       <c r="H86" s="22"/>
-    </row>
-    <row r="87" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I86" s="31"/>
+      <c r="J86" s="22"/>
+    </row>
+    <row r="87" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="16"/>
       <c r="B87" s="31"/>
       <c r="C87" s="22"/>
       <c r="D87" s="22"/>
       <c r="E87" s="16"/>
       <c r="F87" s="22"/>
-      <c r="G87" s="22"/>
+      <c r="G87" s="31"/>
       <c r="H87" s="22"/>
-    </row>
-    <row r="88" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I87" s="31"/>
+      <c r="J87" s="22"/>
+    </row>
+    <row r="88" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="16"/>
       <c r="B88" s="31"/>
       <c r="C88" s="22"/>
       <c r="D88" s="22"/>
       <c r="E88" s="16"/>
       <c r="F88" s="22"/>
-      <c r="G88" s="22"/>
+      <c r="G88" s="31"/>
       <c r="H88" s="22"/>
-    </row>
-    <row r="89" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I88" s="31"/>
+      <c r="J88" s="22"/>
+    </row>
+    <row r="89" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="16"/>
       <c r="B89" s="31"/>
       <c r="C89" s="22"/>
       <c r="D89" s="22"/>
       <c r="E89" s="16"/>
       <c r="F89" s="22"/>
-      <c r="G89" s="22"/>
+      <c r="G89" s="31"/>
       <c r="H89" s="22"/>
-    </row>
-    <row r="90" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I89" s="31"/>
+      <c r="J89" s="22"/>
+    </row>
+    <row r="90" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="16"/>
       <c r="B90" s="31"/>
       <c r="C90" s="22"/>
       <c r="D90" s="22"/>
       <c r="E90" s="16"/>
       <c r="F90" s="22"/>
-      <c r="G90" s="22"/>
+      <c r="G90" s="31"/>
       <c r="H90" s="22"/>
-    </row>
-    <row r="91" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I90" s="31"/>
+      <c r="J90" s="22"/>
+    </row>
+    <row r="91" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="16"/>
       <c r="B91" s="31"/>
       <c r="C91" s="22"/>
       <c r="D91" s="22"/>
       <c r="E91" s="16"/>
       <c r="F91" s="22"/>
-      <c r="G91" s="22"/>
+      <c r="G91" s="31"/>
       <c r="H91" s="22"/>
-    </row>
-    <row r="92" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I91" s="31"/>
+      <c r="J91" s="22"/>
+    </row>
+    <row r="92" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="16"/>
       <c r="B92" s="31"/>
       <c r="C92" s="22"/>
       <c r="D92" s="22"/>
       <c r="E92" s="16"/>
       <c r="F92" s="22"/>
-      <c r="G92" s="22"/>
+      <c r="G92" s="31"/>
       <c r="H92" s="22"/>
-    </row>
-    <row r="93" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I92" s="31"/>
+      <c r="J92" s="22"/>
+    </row>
+    <row r="93" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="16"/>
       <c r="B93" s="31"/>
       <c r="C93" s="22"/>
       <c r="D93" s="22"/>
       <c r="E93" s="16"/>
       <c r="F93" s="22"/>
-      <c r="G93" s="22"/>
+      <c r="G93" s="31"/>
       <c r="H93" s="22"/>
-    </row>
-    <row r="94" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I93" s="31"/>
+      <c r="J93" s="22"/>
+    </row>
+    <row r="94" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="16"/>
       <c r="B94" s="31"/>
       <c r="C94" s="22"/>
       <c r="D94" s="22"/>
       <c r="E94" s="16"/>
       <c r="F94" s="22"/>
-      <c r="G94" s="22"/>
+      <c r="G94" s="31"/>
       <c r="H94" s="22"/>
-    </row>
-    <row r="95" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I94" s="31"/>
+      <c r="J94" s="22"/>
+    </row>
+    <row r="95" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="16"/>
       <c r="B95" s="31"/>
       <c r="C95" s="22"/>
       <c r="D95" s="22"/>
       <c r="E95" s="16"/>
       <c r="F95" s="22"/>
-      <c r="G95" s="22"/>
+      <c r="G95" s="31"/>
       <c r="H95" s="22"/>
-    </row>
-    <row r="96" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I95" s="31"/>
+      <c r="J95" s="22"/>
+    </row>
+    <row r="96" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="16"/>
       <c r="B96" s="31"/>
       <c r="C96" s="22"/>
       <c r="D96" s="22"/>
       <c r="E96" s="16"/>
       <c r="F96" s="22"/>
-      <c r="G96" s="22"/>
+      <c r="G96" s="31"/>
       <c r="H96" s="22"/>
-    </row>
-    <row r="97" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I96" s="31"/>
+      <c r="J96" s="22"/>
+    </row>
+    <row r="97" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="16"/>
       <c r="B97" s="31"/>
       <c r="C97" s="22"/>
       <c r="D97" s="22"/>
       <c r="E97" s="16"/>
       <c r="F97" s="22"/>
-      <c r="G97" s="22"/>
+      <c r="G97" s="31"/>
       <c r="H97" s="22"/>
-    </row>
-    <row r="98" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I97" s="31"/>
+      <c r="J97" s="22"/>
+    </row>
+    <row r="98" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="16"/>
       <c r="B98" s="31"/>
       <c r="C98" s="22"/>
       <c r="D98" s="22"/>
       <c r="E98" s="16"/>
       <c r="F98" s="22"/>
-      <c r="G98" s="22"/>
+      <c r="G98" s="31"/>
       <c r="H98" s="22"/>
-    </row>
-    <row r="99" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I98" s="31"/>
+      <c r="J98" s="22"/>
+    </row>
+    <row r="99" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="16"/>
       <c r="B99" s="31"/>
       <c r="C99" s="22"/>
       <c r="D99" s="22"/>
       <c r="E99" s="16"/>
       <c r="F99" s="22"/>
-      <c r="G99" s="22"/>
+      <c r="G99" s="31"/>
       <c r="H99" s="22"/>
-    </row>
-    <row r="100" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I99" s="31"/>
+      <c r="J99" s="22"/>
+    </row>
+    <row r="100" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="16"/>
       <c r="B100" s="31"/>
       <c r="C100" s="22"/>
       <c r="D100" s="22"/>
       <c r="E100" s="16"/>
       <c r="F100" s="22"/>
-      <c r="G100" s="22"/>
+      <c r="G100" s="31"/>
       <c r="H100" s="22"/>
-    </row>
-    <row r="101" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I100" s="31"/>
+      <c r="J100" s="22"/>
+    </row>
+    <row r="101" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="16"/>
       <c r="B101" s="31"/>
       <c r="C101" s="22"/>
       <c r="D101" s="22"/>
       <c r="E101" s="16"/>
       <c r="F101" s="22"/>
-      <c r="G101" s="22"/>
+      <c r="G101" s="31"/>
       <c r="H101" s="22"/>
-    </row>
-    <row r="102" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I101" s="31"/>
+      <c r="J101" s="22"/>
+    </row>
+    <row r="102" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="16"/>
       <c r="B102" s="31"/>
       <c r="C102" s="22"/>
       <c r="D102" s="22"/>
       <c r="E102" s="16"/>
       <c r="F102" s="22"/>
-      <c r="G102" s="22"/>
+      <c r="G102" s="31"/>
       <c r="H102" s="22"/>
-    </row>
-    <row r="103" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I102" s="31"/>
+      <c r="J102" s="22"/>
+    </row>
+    <row r="103" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="16"/>
       <c r="B103" s="31"/>
       <c r="C103" s="22"/>
       <c r="D103" s="22"/>
       <c r="E103" s="16"/>
       <c r="F103" s="22"/>
-      <c r="G103" s="22"/>
+      <c r="G103" s="31"/>
       <c r="H103" s="22"/>
-    </row>
-    <row r="104" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I103" s="31"/>
+      <c r="J103" s="22"/>
+    </row>
+    <row r="104" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="16"/>
       <c r="B104" s="31"/>
       <c r="C104" s="22"/>
       <c r="D104" s="22"/>
       <c r="E104" s="16"/>
       <c r="F104" s="22"/>
-      <c r="G104" s="22"/>
+      <c r="G104" s="31"/>
       <c r="H104" s="22"/>
-    </row>
-    <row r="105" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I104" s="31"/>
+      <c r="J104" s="22"/>
+    </row>
+    <row r="105" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="16"/>
       <c r="B105" s="31"/>
       <c r="C105" s="22"/>
       <c r="D105" s="22"/>
       <c r="E105" s="16"/>
       <c r="F105" s="22"/>
-      <c r="G105" s="22"/>
+      <c r="G105" s="31"/>
       <c r="H105" s="22"/>
-    </row>
-    <row r="106" spans="1:8" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I105" s="31"/>
+      <c r="J105" s="22"/>
+    </row>
+    <row r="106" spans="1:10" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="16"/>
       <c r="B106" s="31"/>
       <c r="C106" s="22"/>
       <c r="D106" s="22"/>
       <c r="E106" s="16"/>
       <c r="F106" s="22"/>
-      <c r="G106" s="22"/>
+      <c r="G106" s="31"/>
       <c r="H106" s="22"/>
-    </row>
-    <row r="107" spans="1:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I106" s="31"/>
+      <c r="J106" s="22"/>
+    </row>
+    <row r="107" spans="1:10" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="16"/>
       <c r="B107" s="31"/>
       <c r="C107" s="22"/>
       <c r="D107" s="22"/>
       <c r="E107" s="16"/>
       <c r="F107" s="22"/>
-      <c r="G107" s="22"/>
+      <c r="G107" s="31"/>
       <c r="H107" s="22"/>
-    </row>
-    <row r="108" spans="1:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I107" s="31"/>
+      <c r="J107" s="22"/>
+    </row>
+    <row r="108" spans="1:10" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="16"/>
       <c r="B108" s="31"/>
       <c r="C108" s="22"/>
       <c r="D108" s="22"/>
       <c r="E108" s="16"/>
       <c r="F108" s="22"/>
-      <c r="G108" s="22"/>
+      <c r="G108" s="31"/>
       <c r="H108" s="22"/>
-    </row>
-    <row r="109" spans="1:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I108" s="31"/>
+      <c r="J108" s="22"/>
+    </row>
+    <row r="109" spans="1:10" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="16"/>
       <c r="B109" s="31"/>
       <c r="C109" s="22"/>
       <c r="D109" s="22"/>
       <c r="E109" s="16"/>
       <c r="F109" s="22"/>
-      <c r="G109" s="22"/>
+      <c r="G109" s="31"/>
       <c r="H109" s="22"/>
-    </row>
-    <row r="110" spans="1:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I109" s="31"/>
+      <c r="J109" s="22"/>
+    </row>
+    <row r="110" spans="1:10" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="16"/>
       <c r="B110" s="31"/>
       <c r="C110" s="22"/>
       <c r="D110" s="22"/>
       <c r="E110" s="16"/>
       <c r="F110" s="22"/>
-      <c r="G110" s="22"/>
+      <c r="G110" s="31"/>
       <c r="H110" s="22"/>
+      <c r="I110" s="31"/>
+      <c r="J110" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="B1:E3"/>
-    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="J10:J11"/>
     <mergeCell ref="A10:A11"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H5:J5"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="E6:F6"/>

</xml_diff>

<commit_message>
Aimp capacity and correct headers in templates
</commit_message>
<xml_diff>
--- a/src/hydrofia/hydrofia_ph_template.xlsx
+++ b/src/hydrofia/hydrofia_ph_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hydrofia\src\hydrofia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4CDFA7-4295-4239-8A7F-A40C9380475E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9EC8F3-80B3-4159-8ADB-AEF7D583306F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20" yWindow="170" windowWidth="15600" windowHeight="11610" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
   <si>
     <t>Djup</t>
   </si>
@@ -125,16 +125,13 @@
     <t>C</t>
   </si>
   <si>
-    <t>pH-TOT</t>
+    <t>Lab. Temp</t>
   </si>
   <si>
-    <t>labT</t>
+    <t>pH-TOT-labT</t>
   </si>
   <si>
-    <t>25degC</t>
-  </si>
-  <si>
-    <t>Lab. Temp</t>
+    <t>pH-TOT-25</t>
   </si>
 </sst>
 </file>
@@ -971,7 +968,7 @@
     <col min="3" max="3" width="6.54296875" style="3" customWidth="1"/>
     <col min="4" max="6" width="7.81640625" style="3" customWidth="1"/>
     <col min="7" max="7" width="9.81640625" style="3" customWidth="1"/>
-    <col min="8" max="9" width="7.81640625" style="3" customWidth="1"/>
+    <col min="8" max="9" width="13.26953125" style="3" customWidth="1"/>
     <col min="10" max="10" width="12.453125" style="3" customWidth="1"/>
     <col min="11" max="19" width="10.7265625" style="3" customWidth="1"/>
     <col min="20" max="16384" width="28.7265625" style="3"/>
@@ -1832,7 +1829,7 @@
       <c r="I9" s="11"/>
       <c r="J9" s="11"/>
     </row>
-    <row r="10" spans="1:138" s="4" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:138" s="4" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="41" t="s">
         <v>4</v>
       </c>
@@ -1852,13 +1849,13 @@
         <v>12</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J10" s="41" t="s">
         <v>6</v>
@@ -1880,12 +1877,8 @@
       <c r="G11" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I11" s="15" t="s">
-        <v>18</v>
-      </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
       <c r="J11" s="42"/>
     </row>
     <row r="12" spans="1:138" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
From Mosely to Mueller and correct Aimp file
</commit_message>
<xml_diff>
--- a/src/hydrofia/hydrofia_ph_template.xlsx
+++ b/src/hydrofia/hydrofia_ph_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hydrofia\src\hydrofia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D9EC8F3-80B3-4159-8ADB-AEF7D583306F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D463EB1-BE01-4732-A977-EC6D42FB531A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-20" yWindow="170" windowWidth="15600" windowHeight="11610" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -966,7 +966,8 @@
     <col min="1" max="1" width="15.7265625" style="3" customWidth="1"/>
     <col min="2" max="2" width="23.81640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="6.54296875" style="3" customWidth="1"/>
-    <col min="4" max="6" width="7.81640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="10.54296875" style="3" customWidth="1"/>
+    <col min="5" max="6" width="7.81640625" style="3" customWidth="1"/>
     <col min="7" max="7" width="9.81640625" style="3" customWidth="1"/>
     <col min="8" max="9" width="13.26953125" style="3" customWidth="1"/>
     <col min="10" max="10" width="12.453125" style="3" customWidth="1"/>

</xml_diff>